<commit_message>
fix: update documentation structure and adjust chart data for accuracy
</commit_message>
<xml_diff>
--- a/docs/MSTP.xlsx
+++ b/docs/MSTP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish-chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73DBC064-CC80-4D4C-A46A-F84D2D3ED81F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84C6A914-B7E4-44D7-88BE-BB0DED34DBAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
@@ -725,7 +725,7 @@
         <v>11</v>
       </c>
       <c r="H5">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I5">
         <v>23</v>
@@ -734,7 +734,7 @@
         <v>21</v>
       </c>
       <c r="K5">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.4">
@@ -760,7 +760,7 @@
         <v>14</v>
       </c>
       <c r="H6">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I6">
         <v>34</v>
@@ -769,7 +769,7 @@
         <v>31</v>
       </c>
       <c r="K6">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: update performance test documentation and chart data for clarity
</commit_message>
<xml_diff>
--- a/docs/MSTP.xlsx
+++ b/docs/MSTP.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish-chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFD7F321-BF4F-4148-828F-2AA56B0C1595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2656043-13A2-44BE-855F-341D8F0AC390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
   <sheets>
-    <sheet name="3.0.0" sheetId="8" r:id="rId1"/>
-    <sheet name="v2.6.1" sheetId="7" r:id="rId2"/>
-    <sheet name="v2.6.0" sheetId="6" r:id="rId3"/>
-    <sheet name="v2.4.0" sheetId="5" r:id="rId4"/>
-    <sheet name="v2.3.0" sheetId="4" r:id="rId5"/>
-    <sheet name="v2.2.0" sheetId="1" r:id="rId6"/>
-    <sheet name="v2.1.0" sheetId="2" r:id="rId7"/>
-    <sheet name="v2.0.0" sheetId="3" r:id="rId8"/>
+    <sheet name="v3.4.0" sheetId="9" r:id="rId1"/>
+    <sheet name="v3.0.0" sheetId="8" r:id="rId2"/>
+    <sheet name="v2.6.1" sheetId="7" r:id="rId3"/>
+    <sheet name="v2.6.0" sheetId="6" r:id="rId4"/>
+    <sheet name="v2.4.0" sheetId="5" r:id="rId5"/>
+    <sheet name="v2.3.0" sheetId="4" r:id="rId6"/>
+    <sheet name="v2.2.0" sheetId="1" r:id="rId7"/>
+    <sheet name="v2.1.0" sheetId="2" r:id="rId8"/>
+    <sheet name="v2.0.0" sheetId="3" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="39">
   <si>
     <t>Message Count/tick</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -163,6 +164,22 @@
   </si>
   <si>
     <t>200char/Mixed</t>
+  </si>
+  <si>
+    <t>Plain Text</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Styling Only</t>
+  </si>
+  <si>
+    <t>Mention Only (ON)</t>
+  </si>
+  <si>
+    <t>Mention Only (OFF)</t>
+  </si>
+  <si>
+    <t>Mixed</t>
   </si>
 </sst>
 </file>
@@ -545,6 +562,125 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A986CA31-99F9-4BF0-B17F-BAC180A94770}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="19.5" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="24.3984375" customWidth="1"/>
+    <col min="4" max="4" width="22.59765625" customWidth="1"/>
+    <col min="5" max="5" width="21.796875" customWidth="1"/>
+    <col min="6" max="6" width="15.796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A2">
+        <v>50</v>
+      </c>
+      <c r="B2">
+        <v>0.27</v>
+      </c>
+      <c r="C2">
+        <v>0.9</v>
+      </c>
+      <c r="D2">
+        <v>3.06</v>
+      </c>
+      <c r="E2">
+        <v>1.18</v>
+      </c>
+      <c r="F2">
+        <v>1.28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A3">
+        <v>100</v>
+      </c>
+      <c r="B3">
+        <v>1.06</v>
+      </c>
+      <c r="C3">
+        <v>2.16</v>
+      </c>
+      <c r="D3">
+        <v>4.8600000000000003</v>
+      </c>
+      <c r="E3">
+        <v>3.03</v>
+      </c>
+      <c r="F3">
+        <v>2.57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A4">
+        <v>300</v>
+      </c>
+      <c r="B4">
+        <v>3.77</v>
+      </c>
+      <c r="C4">
+        <v>6.93</v>
+      </c>
+      <c r="D4">
+        <v>9.83</v>
+      </c>
+      <c r="E4">
+        <v>8.69</v>
+      </c>
+      <c r="F4">
+        <v>7.06</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A5">
+        <v>500</v>
+      </c>
+      <c r="B5">
+        <v>5.83</v>
+      </c>
+      <c r="C5">
+        <v>10.99</v>
+      </c>
+      <c r="D5">
+        <v>14.27</v>
+      </c>
+      <c r="E5">
+        <v>13</v>
+      </c>
+      <c r="F5">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E78EE54-DA90-4103-8C68-FDEA76202166}">
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -564,7 +700,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>24</v>
@@ -778,7 +914,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D97B426B-7A31-4528-9C0B-EA092DD19299}">
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1012,7 +1148,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80B5C1B6-EB74-483F-9F2C-AFF00761E6BD}">
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1246,7 +1382,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06116B37-F902-49E7-B259-88C657E3068D}">
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1500,7 +1636,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F548A5A-373E-4879-9567-B3774331AE70}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1795,7 +1931,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B38E37E-D8A4-4D05-B5EE-C32E8023EE69}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -2090,7 +2226,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63723110-D812-4C3D-AFC0-E7634718A855}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -2249,7 +2385,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0A4C8FE-4793-4DF4-BD4A-84084E113CBB}">
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>

</xml_diff>